<commit_message>
Reimport master schedule, update JV Puyallup game, add gear store link
- Reimport all team schedules from updated Master Schedule spreadsheet
- Update calendar.html tables, FullCalendar events, and summary stats
- Fix Varsity vs Lakes (Mar 20) in schedule.html after incorrect removal
- JV 3/12 Puyallup: changed from Home/GHHS/4pm to Away/PRC/3:30pm
- C Team stats: corrected home game count for double headers
- Add Tides Gear Store announcement on home page (orders due Mar 13)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Rosters/2026 Teams.xlsx
+++ b/Rosters/2026 Teams.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bsleeter/Documents/Documents - Benjamin's MacBook Pro/Rosters/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bsleeter/Documents/Documents - Benjamin's MacBook Pro/GH Baseball/Rosters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5A185FE-75AD-7E4D-B322-7B73280D9A90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1842BDF7-A1CD-F14E-9F5C-55090652E3E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="940" yWindow="760" windowWidth="28040" windowHeight="17180" xr2:uid="{6C7CCD0D-CDAE-014E-8F59-16CAD8CAA6B6}"/>
+    <workbookView xWindow="920" yWindow="760" windowWidth="28040" windowHeight="17180" xr2:uid="{6C7CCD0D-CDAE-014E-8F59-16CAD8CAA6B6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="60">
   <si>
     <t>Varsity</t>
   </si>
@@ -192,6 +192,30 @@
   </si>
   <si>
     <t>Danny Vorobets</t>
+  </si>
+  <si>
+    <t>Varsity Uniforms</t>
+  </si>
+  <si>
+    <t>Order</t>
+  </si>
+  <si>
+    <t>Small</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Large</t>
+  </si>
+  <si>
+    <t>XL</t>
+  </si>
+  <si>
+    <t>XXL</t>
+  </si>
+  <si>
+    <t>Greyson Riley</t>
   </si>
 </sst>
 </file>
@@ -214,12 +238,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -234,9 +264,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -571,15 +603,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0810B9F6-8C59-7E46-9088-3CA2C090B68A}">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.5" customWidth="1"/>
     <col min="2" max="2" width="17.83203125" customWidth="1"/>
     <col min="3" max="3" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="14.5" customWidth="1"/>
+    <col min="8" max="8" width="14.6640625" customWidth="1"/>
+    <col min="9" max="9" width="16.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -589,9 +624,15 @@
       <c r="C1" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="F1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" t="s">
@@ -600,9 +641,18 @@
       <c r="C2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B3" t="s">
@@ -611,19 +661,37 @@
       <c r="C3" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="F3" s="3">
+        <v>2</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="G4" t="s">
+        <v>54</v>
+      </c>
+      <c r="H4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -633,9 +701,18 @@
       <c r="C5" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B6" t="s">
@@ -644,8 +721,17 @@
       <c r="C6" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -655,53 +741,95 @@
       <c r="C7" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="F7">
+        <v>6</v>
+      </c>
+      <c r="G7" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="2" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="F8">
+        <v>7</v>
+      </c>
+      <c r="G8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C9" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="F9" s="2">
+        <v>8</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>29</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F10">
+        <v>9</v>
+      </c>
+      <c r="G10" t="s">
+        <v>55</v>
+      </c>
+      <c r="H10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>30</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="F11">
+        <v>10</v>
+      </c>
+      <c r="G11" t="s">
+        <v>55</v>
+      </c>
+      <c r="I11" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B12" t="s">
@@ -710,9 +838,18 @@
       <c r="C12" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+      <c r="F12">
+        <v>11</v>
+      </c>
+      <c r="G12" t="s">
+        <v>55</v>
+      </c>
+      <c r="H12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B13" t="s">
@@ -721,19 +858,38 @@
       <c r="C13" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F13">
+        <v>12</v>
+      </c>
+      <c r="G13" t="s">
+        <v>55</v>
+      </c>
+      <c r="I13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C14" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F14">
+        <v>13</v>
+      </c>
+      <c r="G14" t="s">
+        <v>55</v>
+      </c>
+      <c r="H14" t="s">
+        <v>59</v>
+      </c>
+      <c r="I14" s="3"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -743,38 +899,167 @@
       <c r="C15" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F15">
+        <v>14</v>
+      </c>
+      <c r="G15" t="s">
+        <v>56</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>13</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="F16">
+        <v>15</v>
+      </c>
+      <c r="G16" t="s">
+        <v>56</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+      <c r="F17">
+        <v>16</v>
+      </c>
+      <c r="G17" t="s">
+        <v>56</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="F18">
+        <v>17</v>
+      </c>
+      <c r="G18" t="s">
+        <v>56</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="F19">
+        <v>18</v>
+      </c>
+      <c r="G19" t="s">
+        <v>56</v>
+      </c>
+      <c r="H19" t="s">
+        <v>5</v>
+      </c>
+      <c r="I19" s="3"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="F20">
+        <v>19</v>
+      </c>
+      <c r="G20" t="s">
+        <v>56</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>20</v>
+      </c>
+      <c r="F21">
+        <v>20</v>
+      </c>
+      <c r="G21" t="s">
+        <v>56</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F22">
+        <v>21</v>
+      </c>
+      <c r="G22" t="s">
+        <v>57</v>
+      </c>
+      <c r="H22" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F23">
+        <v>22</v>
+      </c>
+      <c r="G23" t="s">
+        <v>57</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F24">
+        <v>23</v>
+      </c>
+      <c r="G24" t="s">
+        <v>57</v>
+      </c>
+      <c r="I24" s="3"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F25">
+        <v>24</v>
+      </c>
+      <c r="G25" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F26">
+        <v>25</v>
+      </c>
+      <c r="G26" t="s">
+        <v>58</v>
+      </c>
+      <c r="I26" s="3"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F27">
+        <v>26</v>
+      </c>
+      <c r="G27" t="s">
+        <v>58</v>
+      </c>
+      <c r="I27" s="3"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="F28">
+        <v>27</v>
+      </c>
+      <c r="G28" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>